<commit_message>
feat(F-NAR-009): EMO.GES / EMO.LEX, ouvertures du monde
Texte seulement. Amorces distinctes, troupe D16.
</commit_message>
<xml_diff>
--- a/stories/arbres/ATOM-EMO.GES.002-02.xlsx
+++ b/stories/arbres/ATOM-EMO.GES.002-02.xlsx
@@ -481,7 +481,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B30"/>
+  <dimension ref="A1:B31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -544,7 +544,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Yanis souffle et fait une pause</t>
+          <t>La tour d'Aniss et le pain chaud</t>
         </is>
       </c>
     </row>
@@ -602,6 +602,11 @@
           <t>secondary_lessons</t>
         </is>
       </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>EMO.LEX.007</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -830,6 +835,18 @@
       <c r="B30" t="inlineStr">
         <is>
           <t>voix-roles-v1</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>fil_rouge</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Aniss veut une tour bien droite. Elle tombe. Il souffle, fait une pause, puis va chercher le pain chaud avec papa.</t>
         </is>
       </c>
     </row>
@@ -1172,7 +1189,7 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Yanis construit une tour dans le salon. La tour tremble. Yanis sent son ventre serré. Papa est près de lui. Tu peux souffler. Tu peux faire une pause. Yanis s'assoit. Il souffle, long et doux. Il fait une pause. Puis il reprend. La tour tient mieux. Plus tard, ils vont à la boulangerie. La file est longue. Yanis sent ses pieds bouger. Il se souvient. Je veux souffler. On fait une pause. Yanis s'assoit sur le banc près de papa. Il souffle. Il fait une pause. Puis il reprend, calme. Même leçon, autre lieu. Souffler aide. Une pause aide.</t>
+          <t>La pluie tapote la vitre du salon. Les gouttes glissent, lentes, une par une. Les manteaux mouillés gouttent près de la porte. Une petite flaque brille sur le carrelage. Dehors, ça sent déjà le pain chaud. Le radiateur fait un tout petit tic. Les chaussures vont ici, Aniss. Je prends une serviette pour les manteaux. Papa aligne les chaussures. Maman essuie une manche encore humide. La maison est un peu froide, ce matin. Le tapis du salon est doux. On peut jouer là. En ce moment, Aniss est sur le tapis. Il a des cubes en bois, lisses et clairs. Les cubes sentent le bois sec. Aniss veut une tour bien droite. Elle va monter très haut. Tu construis avec soin ? Oui, papa. Une grande tour. Je t'écoute depuis la porte. Ça cliquette doucement. Aniss pose un cube. Puis un autre. Les cubes cliquent, tout doux. La tour grandit, un peu penchée. Elle tremble. Un cube glisse. La tour tombe sur le tapis. Ça fait un bruit sourd, dans le salon calme. Aniss sent son ventre se serrer. Sa poitrine va trop vite. Ses mains chauffent. Je suis fâché. C'est trop. La tour est tombée. Tu es fâché. Tu peux souffler, Aniss. Tu peux faire une pause. Aniss s'assoit sur le tapis. Il pose les mains sur ses genoux. Il souffle, long et doux. Une fois. Deux fois. Il fait une pause. Le salon redevient calme. La pluie tapote encore la vitre. Je souffle. Je fais une pause. Bravo. Ton ventre se desserre. Tu as soufflé. Tu as fait une pause. Tu veux reprendre, tout doucement ? Oui. Tout doucement. Aniss reprend un cube. Il le pose sans presser. La tour est petite. Elle tient.</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
@@ -1312,15 +1329,65 @@
       <c r="AV2" s="2" t="inlineStr"/>
       <c r="AW2" t="inlineStr">
         <is>
-          <t>narrateur|Yanis construit une tour dans le salon. La tour tremble. Yanis sent son ventre serré. Papa est près de lui.
-papa|Tu peux souffler. Tu peux faire une pause.
-narrateur|Yanis s'assoit. Il souffle, long et doux. Il fait une pause. Puis il reprend. La tour tient mieux. Plus tard, ils vont à la boulangerie. La file est longue. Yanis sent ses pieds bouger. Il se souvient.
-narrateur|Je veux souffler.
-papa|On fait une pause.
-narrateur|Yanis s'assoit sur le banc près de papa. Il souffle. Il fait une pause. Puis il reprend, calme. Même leçon, autre lieu. Souffler aide. Une pause aide.</t>
-        </is>
-      </c>
-      <c r="AX2" t="inlineStr"/>
+          <t>narrateur|La pluie tapote la vitre du salon.
+narrateur|Les gouttes glissent, lentes, une par une.
+narrateur|Les manteaux mouillés gouttent près de la porte.
+narrateur|Une petite flaque brille sur le carrelage.
+narrateur|Dehors, ça sent déjà le pain chaud.
+narrateur|Le radiateur fait un tout petit tic.
+papa|Les chaussures vont ici, Aniss.
+maman|Je prends une serviette pour les manteaux.
+narrateur|Papa aligne les chaussures.
+narrateur|Maman essuie une manche encore humide.
+maman|La maison est un peu froide, ce matin.
+papa|Le tapis du salon est doux. On peut jouer là.
+narrateur|En ce moment, Aniss est sur le tapis.
+narrateur|Il a des cubes en bois, lisses et clairs.
+narrateur|Les cubes sentent le bois sec.
+narrateur|Aniss veut une tour bien droite.
+enfant-m|Elle va monter très haut.
+papa|Tu construis avec soin ?
+enfant-m|Oui, papa. Une grande tour.
+maman|Je t'écoute depuis la porte. Ça cliquette doucement.
+narrateur|Aniss pose un cube.
+narrateur|Puis un autre.
+narrateur|Les cubes cliquent, tout doux.
+narrateur|La tour grandit, un peu penchée.
+narrateur|Elle tremble.
+narrateur|Un cube glisse.
+narrateur|La tour tombe sur le tapis.
+narrateur|Ça fait un bruit sourd, dans le salon calme.
+narrateur|Aniss sent son ventre se serrer.
+narrateur|Sa poitrine va trop vite.
+narrateur|Ses mains chauffent.
+enfant-m|Je suis fâché. C'est trop.
+maman|La tour est tombée. Tu es fâché.
+papa|Tu peux souffler, Aniss.
+papa|Tu peux faire une pause.
+narrateur|Aniss s'assoit sur le tapis.
+narrateur|Il pose les mains sur ses genoux.
+narrateur|Il souffle, long et doux.
+narrateur|Une fois.
+narrateur|Deux fois.
+narrateur|Il fait une pause.
+narrateur|Le salon redevient calme.
+narrateur|La pluie tapote encore la vitre.
+enfant-m|Je souffle. Je fais une pause.
+maman|Bravo. Ton ventre se desserre.
+papa|Tu as soufflé. Tu as fait une pause.
+papa|Tu veux reprendre, tout doucement ?
+enfant-m|Oui. Tout doucement.
+narrateur|Aniss reprend un cube.
+narrateur|Il le pose sans presser.
+narrateur|La tour est petite.
+narrateur|Elle tient.</t>
+        </is>
+      </c>
+      <c r="AX2" t="inlineStr">
+        <is>
+          <t>pluie,cubes_bois</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -1345,7 +1412,7 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>Yanis sent son corps trop plein. Que fait-il ?</t>
+          <t>Aniss sent son corps trop plein. Que fait-il ?</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
@@ -1501,7 +1568,8 @@
       </c>
       <c r="AW3" t="inlineStr">
         <is>
-          <t>narrateur|Yanis sent son corps trop plein. Que fait-il ?</t>
+          <t>narrateur|Aniss sent son corps trop plein.
+narrateur|Que fait-il ?</t>
         </is>
       </c>
       <c r="AX3" t="inlineStr"/>
@@ -1529,7 +1597,7 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Yanis a soufflé. Il a fait une pause. Dans le salon, puis à la boulangerie.</t>
+          <t>Aniss a soufflé. Il a fait une pause. Plus tard, la pluie devient fine. On va chercher le pain ? Prenez le sac. Il est près de la porte. Oui. Le pain chaud. Aniss et papa marchent sous le ciel gris. Les gouttes font des ronds dans les flaques. La boulangerie sent le beurre et la farine. La file est longue. Aniss sent ses pieds bouger. Son ventre se serre un peu. C'est trop. J'attends. Je suis fâché. Tu te souviens, Aniss ? Tu peux souffler. Tu peux faire une pause. Aniss s'assoit sur le banc, près de papa. Il souffle, long et doux. Il fait une pause. Ses pieds se posent. Je souffle. Je fais une pause. Bravo. Tu as repris, calme. La file avance. Le pain arrive, encore tiède.</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
@@ -1673,10 +1741,36 @@
       </c>
       <c r="AW4" t="inlineStr">
         <is>
-          <t>narrateur|Yanis a soufflé. Il a fait une pause. Dans le salon, puis à la boulangerie.</t>
-        </is>
-      </c>
-      <c r="AX4" t="inlineStr"/>
+          <t>narrateur|Aniss a soufflé.
+narrateur|Il a fait une pause.
+narrateur|Plus tard, la pluie devient fine.
+papa|On va chercher le pain ?
+maman|Prenez le sac. Il est près de la porte.
+enfant-m|Oui. Le pain chaud.
+narrateur|Aniss et papa marchent sous le ciel gris.
+narrateur|Les gouttes font des ronds dans les flaques.
+narrateur|La boulangerie sent le beurre et la farine.
+narrateur|La file est longue.
+narrateur|Aniss sent ses pieds bouger.
+narrateur|Son ventre se serre un peu.
+enfant-m|C'est trop. J'attends. Je suis fâché.
+papa|Tu te souviens, Aniss ?
+papa|Tu peux souffler. Tu peux faire une pause.
+narrateur|Aniss s'assoit sur le banc, près de papa.
+narrateur|Il souffle, long et doux.
+narrateur|Il fait une pause.
+narrateur|Ses pieds se posent.
+enfant-m|Je souffle. Je fais une pause.
+papa|Bravo. Tu as repris, calme.
+narrateur|La file avance.
+narrateur|Le pain arrive, encore tiède.</t>
+        </is>
+      </c>
+      <c r="AX4" t="inlineStr">
+        <is>
+          <t>pluie,boulangerie</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -1701,7 +1795,7 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Yanis tient le pain. Papa sourit.</t>
+          <t>Aniss tient le pain encore tiède. Le papier craque un peu entre ses mains. Tu as attendu. Tu as soufflé. Tu as fait du bon travail. Le pain est chaud, papa. On rentre le montrer à maman ? Oui. Ils marchent. La pluie est fine. Aniss serre le pain contre son manteau. La maison n'est plus très loin.</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
@@ -1837,10 +1931,23 @@
       <c r="AV5" s="2" t="inlineStr"/>
       <c r="AW5" t="inlineStr">
         <is>
-          <t>narrateur|Yanis tient le pain. Papa sourit.</t>
-        </is>
-      </c>
-      <c r="AX5" t="inlineStr"/>
+          <t>narrateur|Aniss tient le pain encore tiède.
+narrateur|Le papier craque un peu entre ses mains.
+papa|Tu as attendu. Tu as soufflé.
+papa|Tu as fait du bon travail.
+enfant-m|Le pain est chaud, papa.
+papa|On rentre le montrer à maman ?
+enfant-m|Oui.
+narrateur|Ils marchent. La pluie est fine.
+narrateur|Aniss serre le pain contre son manteau.
+narrateur|La maison n'est plus très loin.</t>
+        </is>
+      </c>
+      <c r="AX5" t="inlineStr">
+        <is>
+          <t>pluie,papier</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -1865,7 +1972,7 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>L'histoire est finie.</t>
+          <t>J'ai soufflé. J'ai fait une pause. Bravo, Aniss. Le pain est là. Vous voilà. Ça sent bon, tout le salon. L'histoire est finie.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
@@ -2005,7 +2112,11 @@
       <c r="AV6" s="2" t="inlineStr"/>
       <c r="AW6" t="inlineStr">
         <is>
-          <t>narrateur|L'histoire est finie.</t>
+          <t>enfant-m|J'ai soufflé. J'ai fait une pause.
+papa|Bravo, Aniss.
+maman|Le pain est là. Vous voilà.
+maman|Ça sent bon, tout le salon.
+narrateur|L'histoire est finie.</t>
         </is>
       </c>
       <c r="AX6" t="inlineStr"/>
@@ -2027,7 +2138,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A5"/>
+  <dimension ref="A1:A6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -2065,6 +2176,13 @@
       <c r="A5" t="inlineStr">
         <is>
           <t>F-AUD-007 colonne sons ; vide = silence ; jamais parler dans le bruit</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>F-NAR-009 ouverture du monde, fusion agents</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(F-NAR-019): ATOM-EMO.GES.002-02 Aniss souffle et fait une pause
</commit_message>
<xml_diff>
--- a/stories/arbres/ATOM-EMO.GES.002-02.xlsx
+++ b/stories/arbres/ATOM-EMO.GES.002-02.xlsx
@@ -544,7 +544,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>La tour d'Aniss et le pain chaud</t>
+          <t>Aniss souffle et fait une pause</t>
         </is>
       </c>
     </row>
@@ -671,7 +671,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>salon puis boulangerie</t>
+          <t>salon, fenêtre, cubes, bois, soleil, pain, boulangerie, comptoir, file, papier</t>
         </is>
       </c>
     </row>
@@ -841,7 +841,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Aniss veut une tour bien droite. Elle tombe. Il souffle, fait une pause, puis va chercher le pain chaud avec papa.</t>
+          <t>Un air de pain chaud glisse dans le salon. Près de la fenêtre, un éclat de comptoir brille. Aniss veut la tour maintenant. Elle tremble. Ventre serré, sourire parti, papa accroupi. Il souffle, pause. Merci vécu. Deuxième ruse à la boulangerie. Un éclat de comptoir tient sur le bois.</t>
         </is>
       </c>
     </row>
@@ -1184,17 +1184,17 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>La pluie tapote la vitre du salon. Les gouttes glissent, lentes, une par une. Les manteaux mouillés gouttent près de la porte. Une petite flaque brille sur le carrelage. Dehors, ça sent déjà le pain chaud. Le radiateur fait un tout petit tic. Les chaussures vont ici, Aniss. Je prends une serviette pour les manteaux. Papa aligne les chaussures. Maman essuie une manche encore humide. La maison est un peu froide, ce matin. Le tapis du salon est doux. On peut jouer là. En ce moment, Aniss est sur le tapis. Il a des cubes en bois, lisses et clairs. Les cubes sentent le bois sec. Aniss veut une tour bien droite. Elle va monter très haut. Tu construis avec soin ? Oui, papa. Une grande tour. Je t'écoute depuis la porte. Ça cliquette doucement. Aniss pose un cube. Puis un autre. Les cubes cliquent, tout doux. La tour grandit, un peu penchée. Elle tremble. Un cube glisse. La tour tombe sur le tapis. Ça fait un bruit sourd, dans le salon calme. Aniss sent son ventre se serrer. Sa poitrine va trop vite. Ses mains chauffent. Je suis fâché. C'est trop. La tour est tombée. Tu es fâché. Tu peux souffler, Aniss. Tu peux faire une pause. Aniss s'assoit sur le tapis. Il pose les mains sur ses genoux. Il souffle, long et doux. Une fois. Deux fois. Il fait une pause. Le salon redevient calme. La pluie tapote encore la vitre. Je souffle. Je fais une pause. Bravo. Ton ventre se desserre. Tu as soufflé. Tu as fait une pause. Tu veux reprendre, tout doucement ? Oui. Tout doucement. Aniss reprend un cube. Il le pose sans presser. La tour est petite. Elle tient.</t>
+          <t>Un air de pain chaud glisse dans le salon. Ça sent le pain, papa. Tu le sens, le pain, Aniss ? Oui, papa. Le soleil tient les cubes, près du bois. Les cubes sont lisses, un peu froids. Ils sont froids, maman. Tu les touches, les cubes ? Oui, maman. Près de la fenêtre, un éclat de comptoir brille. Il brille, papa. Tu le vois, le petit point ? Oui, un petit point. La boulangerie est là, de l'autre côté. Le pain est là-bas. On ira chercher le pain, plus tard. Oui. La tour, d'abord ? La tour, maintenant ! Le bois sent le soleil. Il est chaud. Le bois, sous tes mains ? Oui. En ce moment, Aniss prend un cube. Il veut une tour, très haute. Tout de suite. Elle va monter. Il pose un cube sur le bois. Puis un autre, trop vite. Tu poses les cubes, Aniss ? Oui, papa. Tes mains vont vite, Aniss ? Un peu, maman. La tour grandit, un peu penchée. Elle tremble sur le bois. Un cube glisse. La tour tombe, sourdement. Oh. Aniss tremble un peu. Son ventre se serre. Le sourire d'Aniss disparaît. C'est trop, papa. Tu vois la tour, Aniss ? Oui, papa. Tes épaules sont hautes, Aniss ? Un peu, maman. Papa s'accroupit à la même hauteur. Aniss regarde papa. L'éclat de comptoir tremble, puis tient.</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>La pluie tapote la vitre du salon. Les gouttes glissent, lentes, une par une. Les manteaux mouillés gouttent près de la porte. Une petite flaque brille sur le carrelage. Dehors, ça sent déjà le pain chaud. Le radiateur fait un tout petit tic. Les chaussures vont ici, Aniss. Je prends une serviette pour les manteaux. Papa aligne les chaussures. Maman essuie une manche encore humide. La maison est un peu froide, ce matin. Le tapis du salon est doux. On peut jouer là. En ce moment, Aniss est sur le tapis. Il a des cubes en bois, lisses et clairs. Les cubes sentent le bois sec. Aniss veut une tour bien droite. Elle va monter très haut. Tu construis avec soin ? Oui, papa. Une grande tour. Je t'écoute depuis la porte. Ça cliquette doucement. Aniss pose un cube. Puis un autre. Les cubes cliquent, tout doux. La tour grandit, un peu penchée. Elle tremble. Un cube glisse. La tour tombe sur le tapis. Ça fait un bruit sourd, dans le salon calme. Aniss sent son ventre se serrer. Sa poitrine va trop vite. Ses mains chauffent. Je suis fâché. C'est trop. La tour est tombée. Tu es fâché. Tu peux souffler, Aniss. Tu peux faire une pause. Aniss s'assoit sur le tapis. Il pose les mains sur ses genoux. Il souffle, long et doux. Une fois. Deux fois. Il fait une pause. Le salon redevient calme. La pluie tapote encore la vitre. Je souffle. Je fais une pause. Bravo. Ton ventre se desserre. Tu as soufflé. Tu as fait une pause. Tu veux reprendre, tout doucement ? Oui. Tout doucement. Aniss reprend un cube. Il le pose sans presser. La tour est petite. Elle tient.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Un air de pain chaud glisse dans le salon. Ça sent le pain, papa. Tu le sens, le pain, Aniss ? Oui, papa. Le soleil tient les cubes, près du bois. Les cubes sont lisses, un peu froids. Ils sont froids, maman. Tu les touches, les cubes ? Oui, maman. Près de la fenêtre, un &lt;emphasis level="moderate"&gt;éclat de comptoir&lt;/emphasis&gt; brille. Il brille, papa. Tu le vois, le petit point ? Oui, un petit point. La boulangerie est là, de l'autre côté. Le pain est là-bas. On ira chercher le pain, plus tard. Oui. La tour, d'abord ? La tour, maintenant ! Le bois sent le soleil. Il est chaud. Le bois, sous tes mains ? Oui. En ce moment, Aniss prend un cube. Il veut une tour, très haute. Tout de suite. Elle va monter. Il pose un cube sur le bois. Puis un autre, trop vite. Tu poses les cubes, Aniss ? Oui, papa. Tes mains vont vite, Aniss ? Un peu, maman. La tour grandit, un peu penchée. Elle tremble sur le bois. Un cube glisse. La tour tombe, sourdement. Oh. Aniss tremble un peu. Son ventre se serre. Le sourire d'Aniss disparaît. C'est trop, papa. Tu vois la tour, Aniss ? Oui, papa. Tes épaules sont hautes, Aniss ? Un peu, maman. Papa s'accroupit à la même hauteur. Aniss regarde papa. L'éclat de comptoir tremble, puis tient.&lt;/prosody&gt;&lt;break time="500ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Yanis construit une tour dans le salon. La tour tremble. Yanis sent son ventre serré. Papa est près de lui. Papa dit : tu peux &lt;emphasis&gt;souffler&lt;/emphasis&gt;. Tu peux faire une pause. Yanis s'assoit. Il souffle, long et doux. Il fait une pause. Puis il reprend. La tour tient mieux. Plus tard, ils vont à la boulangerie. La file est longue. Yanis sent ses pieds bouger. Il se souvient. Il dit : je veux souffler. Papa dit : on fait une pause. Yanis s'assoit sur le banc près de papa. Il souffle. Il fait une pause. Puis il reprend, calme. Même leçon, autre lieu. Souffler aide. Une pause aide. [pause]</t>
+          <t>Un air de pain chaud glisse dans le salon. Ça sent le pain, papa. Tu le sens, le pain, Aniss ? Oui, papa. Le soleil tient les cubes, près du bois. Les cubes sont lisses, un peu froids. Ils sont froids, maman. Tu les touches, les cubes ? Oui, maman. Près de la fenêtre, un &lt;emphasis&gt;éclat de comptoir&lt;/emphasis&gt; brille. Il brille, papa. Tu le vois, le petit point ? Oui, un petit point. La boulangerie est là, de l'autre côté. Le pain est là-bas. On ira chercher le pain, plus tard. Oui. La tour, d'abord ? La tour, maintenant ! Le bois sent le soleil. Il est chaud. Le bois, sous tes mains ? Oui. En ce moment, Aniss prend un cube. Il veut une tour, très haute. Tout de suite. Elle va monter. Il pose un cube sur le bois. Puis un autre, trop vite. Tu poses les cubes, Aniss ? Oui, papa. Tes mains vont vite, Aniss ? Un peu, maman. La tour grandit, un peu penchée. Elle tremble sur le bois. Un cube glisse. La tour tombe, sourdement. Oh. Aniss tremble un peu. Son ventre se serre. Le sourire d'Aniss disparaît. C'est trop, papa. Tu vois la tour, Aniss ? Oui, papa. Tes épaules sont hautes, Aniss ? Un peu, maman. Papa s'accroupit à la même hauteur. Aniss regarde papa. L'éclat de comptoir tremble, puis tient. [pause]</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr"/>
@@ -1241,7 +1241,7 @@
         </is>
       </c>
       <c r="Y2" s="2" t="n">
-        <v>148</v>
+        <v>142</v>
       </c>
       <c r="Z2" s="2" t="inlineStr">
         <is>
@@ -1249,7 +1249,7 @@
         </is>
       </c>
       <c r="AA2" s="2" t="n">
-        <v>0.96</v>
+        <v>0.98</v>
       </c>
       <c r="AB2" s="2" t="n">
         <v>1.12</v>
@@ -1275,30 +1275,30 @@
       </c>
       <c r="AH2" s="2" t="inlineStr">
         <is>
-          <t>souffler</t>
+          <t>éclat de comptoir</t>
         </is>
       </c>
       <c r="AI2" s="2" t="n">
         <v>0</v>
       </c>
       <c r="AJ2" s="2" t="n">
-        <v>400</v>
+        <v>500</v>
       </c>
       <c r="AK2" s="2" t="n">
-        <v>280</v>
+        <v>260</v>
       </c>
       <c r="AL2" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>warm</t>
         </is>
       </c>
       <c r="AM2" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>storytelling</t>
         </is>
       </c>
       <c r="AN2" s="2" t="n">
-        <v>0.333</v>
+        <v>0.36</v>
       </c>
       <c r="AO2" s="2" t="inlineStr"/>
       <c r="AP2" s="2" t="inlineStr">
@@ -1307,10 +1307,10 @@
         </is>
       </c>
       <c r="AQ2" s="2" t="n">
-        <v>0.96</v>
+        <v>0.98</v>
       </c>
       <c r="AR2" s="2" t="n">
-        <v>0.96</v>
+        <v>0.98</v>
       </c>
       <c r="AS2" s="2" t="n">
         <v>100</v>
@@ -1321,66 +1321,67 @@
       <c r="AU2" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="AV2" s="2" t="inlineStr"/>
+      <c r="AV2" s="2" t="inlineStr">
+        <is>
+          <t>arc=installation; intention=émerveiller puis tendre; emotion=impatience puis trop_plein; intensite=2; destinataire=enfant; sous_texte=il_veut_la_tour_maintenant; tempo=naturel puis resserré; sourire=léger puis aucun; respiration=ample puis retenue</t>
+        </is>
+      </c>
       <c r="AW2" t="inlineStr">
         <is>
-          <t>narrateur|La pluie tapote la vitre du salon.
-narrateur|Les gouttes glissent, lentes, une par une.
-narrateur|Les manteaux mouillés gouttent près de la porte.
-narrateur|Une petite flaque brille sur le carrelage.
-narrateur|Dehors, ça sent déjà le pain chaud.
-narrateur|Le radiateur fait un tout petit tic.
-papa|Les chaussures vont ici, Aniss.
-maman|Je prends une serviette pour les manteaux.
-narrateur|Papa aligne les chaussures.
-narrateur|Maman essuie une manche encore humide.
-maman|La maison est un peu froide, ce matin.
-papa|Le tapis du salon est doux. On peut jouer là.
-narrateur|En ce moment, Aniss est sur le tapis.
-narrateur|Il a des cubes en bois, lisses et clairs.
-narrateur|Les cubes sentent le bois sec.
-narrateur|Aniss veut une tour bien droite.
-enfant-m|Elle va monter très haut.
-papa|Tu construis avec soin ?
-enfant-m|Oui, papa. Une grande tour.
-maman|Je t'écoute depuis la porte. Ça cliquette doucement.
-narrateur|Aniss pose un cube.
-narrateur|Puis un autre.
-narrateur|Les cubes cliquent, tout doux.
+          <t>narrateur|Un air de pain chaud glisse dans le salon.
+enfant-m|Ça sent le pain, papa.
+papa|Tu le sens, le pain, Aniss ?
+enfant-m|Oui, papa.
+narrateur|Le soleil tient les cubes, près du bois.
+narrateur|Les cubes sont lisses, un peu froids.
+enfant-m|Ils sont froids, maman.
+maman|Tu les touches, les cubes ?
+enfant-m|Oui, maman.
+narrateur|Près de la fenêtre, un éclat de comptoir brille.
+enfant-m|Il brille, papa.
+papa|Tu le vois, le petit point ?
+enfant-m|Oui, un petit point.
+narrateur|La boulangerie est là, de l'autre côté.
+enfant-m|Le pain est là-bas.
+maman|On ira chercher le pain, plus tard.
+enfant-m|Oui.
+papa|La tour, d'abord ?
+enfant-m|La tour, maintenant !
+narrateur|Le bois sent le soleil.
+enfant-m|Il est chaud.
+papa|Le bois, sous tes mains ?
+enfant-m|Oui.
+narrateur|En ce moment, Aniss prend un cube.
+narrateur|Il veut une tour, très haute.
+enfant-m|Tout de suite.
+enfant-m|Elle va monter.
+narrateur|Il pose un cube sur le bois.
+narrateur|Puis un autre, trop vite.
+papa|Tu poses les cubes, Aniss ?
+enfant-m|Oui, papa.
+maman|Tes mains vont vite, Aniss ?
+enfant-m|Un peu, maman.
 narrateur|La tour grandit, un peu penchée.
-narrateur|Elle tremble.
+narrateur|Elle tremble sur le bois.
 narrateur|Un cube glisse.
-narrateur|La tour tombe sur le tapis.
-narrateur|Ça fait un bruit sourd, dans le salon calme.
-narrateur|Aniss sent son ventre se serrer.
-narrateur|Sa poitrine va trop vite.
-narrateur|Ses mains chauffent.
-enfant-m|Je suis fâché. C'est trop.
-maman|La tour est tombée. Tu es fâché.
-papa|Tu peux souffler, Aniss.
-papa|Tu peux faire une pause.
-narrateur|Aniss s'assoit sur le tapis.
-narrateur|Il pose les mains sur ses genoux.
-narrateur|Il souffle, long et doux.
-narrateur|Une fois.
-narrateur|Deux fois.
-narrateur|Il fait une pause.
-narrateur|Le salon redevient calme.
-narrateur|La pluie tapote encore la vitre.
-enfant-m|Je souffle. Je fais une pause.
-maman|Bravo. Ton ventre se desserre.
-papa|Tu as soufflé. Tu as fait une pause.
-papa|Tu veux reprendre, tout doucement ?
-enfant-m|Oui. Tout doucement.
-narrateur|Aniss reprend un cube.
-narrateur|Il le pose sans presser.
-narrateur|La tour est petite.
-narrateur|Elle tient.</t>
+narrateur|La tour tombe, sourdement.
+enfant-m|Oh.
+narrateur|Aniss tremble un peu.
+narrateur|Son ventre se serre.
+narrateur|Le sourire d'Aniss disparaît.
+enfant-m|C'est trop, papa.
+papa|Tu vois la tour, Aniss ?
+enfant-m|Oui, papa.
+maman|Tes épaules sont hautes, Aniss ?
+enfant-m|Un peu, maman.
+narrateur|Papa s'accroupit à la même hauteur.
+narrateur|Aniss regarde papa.
+narrateur|L'éclat de comptoir tremble, puis tient.</t>
         </is>
       </c>
       <c r="AX2" t="inlineStr">
         <is>
-          <t>pluie,cubes_bois</t>
+          <t>fenetre</t>
         </is>
       </c>
     </row>
@@ -1412,12 +1413,12 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Aniss sent son corps trop plein. Que fait-il ?</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;&lt;emphasis level="moderate"&gt;Aniss&lt;/emphasis&gt; sent son corps trop plein. Que fait-il ?&lt;/prosody&gt;&lt;break time="700ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>Yanis sent son corps trop plein. Que fait-il ?</t>
+          <t>&lt;soft&gt;&lt;slow&gt;&lt;emphasis&gt;Aniss&lt;/emphasis&gt; sent son corps trop plein. Que fait-il ?&lt;/slow&gt;&lt;/soft&gt; [pause]</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -1480,18 +1481,18 @@
         </is>
       </c>
       <c r="Y3" s="2" t="n">
-        <v>130</v>
+        <v>120</v>
       </c>
       <c r="Z3" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>slow</t>
         </is>
       </c>
       <c r="AA3" s="2" t="n">
-        <v>0.9</v>
+        <v>0.86</v>
       </c>
       <c r="AB3" s="2" t="n">
-        <v>1.24</v>
+        <v>1.27</v>
       </c>
       <c r="AC3" s="2" t="inlineStr">
         <is>
@@ -1506,34 +1507,38 @@
       <c r="AE3" s="2" t="inlineStr"/>
       <c r="AF3" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>soft</t>
         </is>
       </c>
       <c r="AG3" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="AH3" s="2" t="inlineStr"/>
+        <v>-2</v>
+      </c>
+      <c r="AH3" s="2" t="inlineStr">
+        <is>
+          <t>Aniss</t>
+        </is>
+      </c>
       <c r="AI3" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ3" s="2" t="n">
-        <v>250</v>
+        <v>700</v>
       </c>
       <c r="AK3" s="2" t="n">
-        <v>280</v>
+        <v>320</v>
       </c>
       <c r="AL3" s="2" t="inlineStr">
         <is>
-          <t>warm</t>
+          <t>focused</t>
         </is>
       </c>
       <c r="AM3" s="2" t="inlineStr">
         <is>
-          <t>rise</t>
+          <t>rising</t>
         </is>
       </c>
       <c r="AN3" s="2" t="n">
-        <v>0.333</v>
+        <v>0.32</v>
       </c>
       <c r="AO3" s="2" t="inlineStr"/>
       <c r="AP3" s="2" t="inlineStr">
@@ -1542,23 +1547,23 @@
         </is>
       </c>
       <c r="AQ3" s="2" t="n">
-        <v>0.9</v>
+        <v>0.86</v>
       </c>
       <c r="AR3" s="2" t="n">
-        <v>0.9</v>
+        <v>0.86</v>
       </c>
       <c r="AS3" s="2" t="n">
-        <v>100</v>
+        <v>82</v>
       </c>
       <c r="AT3" s="2" t="n">
         <v>50</v>
       </c>
       <c r="AU3" s="2" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="AV3" s="2" t="inlineStr">
         <is>
-          <t>question d'écoute, ne change pas le cours</t>
+          <t>arc=indice; intention=faire_deviner; emotion=attention; intensite=1; destinataire=enfant; sous_texte=corps_trop_plein_que_fait_il; tempo=suspendu; sourire=aucun; respiration=courte_avant_question</t>
         </is>
       </c>
       <c r="AW3" t="inlineStr">
@@ -1591,17 +1596,17 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Aniss a soufflé. Il a fait une pause. Plus tard, la pluie devient fine. On va chercher le pain ? Prenez le sac. Il est près de la porte. Oui. Le pain chaud. Aniss et papa marchent sous le ciel gris. Les gouttes font des ronds dans les flaques. La boulangerie sent le beurre et la farine. La file est longue. Aniss sent ses pieds bouger. Son ventre se serre un peu. C'est trop. J'attends. Je suis fâché. Tu te souviens, Aniss ? Tu peux souffler. Tu peux faire une pause. Aniss s'assoit sur le banc, près de papa. Il souffle, long et doux. Il fait une pause. Ses pieds se posent. Je souffle. Je fais une pause. Bravo. Tu as repris, calme. La file avance. Le pain arrive, encore tiède.</t>
+          <t>Aniss veut la tour, maintenant. Tout de suite ! Il pose les cubes trop vite. La tour penche, puis tombe. Son ventre reste serré. Le sourire ne revient pas. Oh. Aniss s'assoit près du bois. Il pose les mains sur ses genoux. Il souffle, un filet d'air. L'air sort, long. Il fait une pause. Tu restes près de nous, Aniss ? Je reste ici, papa ? On s'assoit, puis on regarde. D'accord. Aniss reste un moment, les mains ouvertes. Sa poitrine descend, plus lente. Merci, Aniss. Papa a vu les deux, près des cubes. Le bois est tiède, sous les doigts. Il est chaud. Aniss reprend un cube, sans se presser. Sans me presser. Il tient, là ? Oui, là. La tour est petite. Elle tient sur le bois. Tes mains sont au chaud, Aniss ? Un peu, maman. On va au pain ? Le sac est près de la porte ? Oui, maman. Tu prends le sac, Aniss ? Oui, papa. Aniss glisse la main sur le bois. Le petit point. Il brille, là ? Oui, là. Aniss pose les mains sur le bois. Il reste, sans se presser.</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Aniss a soufflé. Il a fait une pause. Plus tard, la pluie devient fine. On va chercher le pain ? Prenez le sac. Il est près de la porte. Oui. Le pain chaud. Aniss et papa marchent sous le ciel gris. Les gouttes font des ronds dans les flaques. La boulangerie sent le beurre et la farine. La file est longue. Aniss sent ses pieds bouger. Son ventre se serre un peu. C'est trop. J'attends. Je suis fâché. Tu te souviens, Aniss ? Tu peux souffler. Tu peux faire une pause. Aniss s'assoit sur le banc, près de papa. Il souffle, long et doux. Il fait une pause. Ses pieds se posent. Je souffle. Je fais une pause. Bravo. Tu as repris, calme. La file avance. Le pain arrive, encore tiède.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Aniss veut la tour, maintenant. Tout de suite ! Il pose les cubes trop vite. La tour penche, puis tombe. Son ventre reste serré. Le sourire ne revient pas. Oh. Aniss s'assoit près du bois. Il pose les mains sur ses genoux. Il &lt;emphasis level="moderate"&gt;souffle&lt;/emphasis&gt;, un filet d'air. L'air sort, long. Il fait une pause. Tu restes près de nous, Aniss ? Je reste ici, papa ? On s'assoit, puis on regarde. D'accord. Aniss reste un moment, les mains ouvertes. Sa poitrine descend, plus lente. Merci, Aniss. Papa a vu les deux, près des cubes. Le bois est tiède, sous les doigts. Il est chaud. Aniss reprend un cube, sans se presser. Sans me presser. Il tient, là ? Oui, là. La tour est petite. Elle tient sur le bois. Tes mains sont au chaud, Aniss ? Un peu, maman. On va au pain ? Le sac est près de la porte ? Oui, maman. Tu prends le sac, Aniss ? Oui, papa. Aniss glisse la main sur le bois. Le petit point. Il brille, là ? Oui, là. Aniss pose les mains sur le bois. Il reste, sans se presser.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>Yanis a soufflé. Il a fait une &lt;emphasis&gt;pause&lt;/emphasis&gt;. Dans le salon, puis à la boulangerie. [pause]</t>
+          <t>Aniss veut la tour, maintenant. Tout de suite ! Il pose les cubes trop vite. La tour penche, puis tombe. Son ventre reste serré. Le sourire ne revient pas. Oh. Aniss s'assoit près du bois. Il pose les mains sur ses genoux. Il &lt;emphasis&gt;souffle&lt;/emphasis&gt;, un filet d'air. L'air sort, long. Il fait une pause. Tu restes près de nous, Aniss ? Je reste ici, papa ? On s'assoit, puis on regarde. D'accord. Aniss reste un moment, les mains ouvertes. Sa poitrine descend, plus lente. Merci, Aniss. Papa a vu les deux, près des cubes. Le bois est tiède, sous les doigts. Il est chaud. Aniss reprend un cube, sans se presser. Sans me presser. Il tient, là ? Oui, là. La tour est petite. Elle tient sur le bois. Tes mains sont au chaud, Aniss ? Un peu, maman. On va au pain ? Le sac est près de la porte ? Oui, maman. Tu prends le sac, Aniss ? Oui, papa. Aniss glisse la main sur le bois. Le petit point. Il brille, là ? Oui, là. Aniss pose les mains sur le bois. Il reste, sans se presser. [pause]</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr"/>
@@ -1648,7 +1653,7 @@
         </is>
       </c>
       <c r="Y4" s="2" t="n">
-        <v>148</v>
+        <v>140</v>
       </c>
       <c r="Z4" s="2" t="inlineStr">
         <is>
@@ -1656,10 +1661,10 @@
         </is>
       </c>
       <c r="AA4" s="2" t="n">
-        <v>0.96</v>
+        <v>0.97</v>
       </c>
       <c r="AB4" s="2" t="n">
-        <v>1.12</v>
+        <v>1.14</v>
       </c>
       <c r="AC4" s="2" t="inlineStr">
         <is>
@@ -1682,30 +1687,30 @@
       </c>
       <c r="AH4" s="2" t="inlineStr">
         <is>
-          <t>pause</t>
+          <t>souffle</t>
         </is>
       </c>
       <c r="AI4" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ4" s="2" t="n">
-        <v>450</v>
+        <v>560</v>
       </c>
       <c r="AK4" s="2" t="n">
-        <v>280</v>
+        <v>270</v>
       </c>
       <c r="AL4" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>bright</t>
         </is>
       </c>
       <c r="AM4" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN4" s="2" t="n">
-        <v>0.333</v>
+        <v>0.35</v>
       </c>
       <c r="AO4" s="2" t="inlineStr"/>
       <c r="AP4" s="2" t="inlineStr">
@@ -1714,10 +1719,10 @@
         </is>
       </c>
       <c r="AQ4" s="2" t="n">
-        <v>0.96</v>
+        <v>0.97</v>
       </c>
       <c r="AR4" s="2" t="n">
-        <v>0.96</v>
+        <v>0.97</v>
       </c>
       <c r="AS4" s="2" t="n">
         <v>100</v>
@@ -1730,39 +1735,57 @@
       </c>
       <c r="AV4" s="2" t="inlineStr">
         <is>
-          <t>confirmation ; le moteur peut dire engine_ok/near avant ce chunk</t>
+          <t>arc=résolution; intention=faire_vivre_le_geste; emotion=trop_plein puis fierté_calme; intensite=2; destinataire=enfant; sous_texte=il_souffle_il_fait_une_pause; tempo=naturel; sourire=léger; respiration=relâchée</t>
         </is>
       </c>
       <c r="AW4" t="inlineStr">
         <is>
-          <t>narrateur|Aniss a soufflé.
-narrateur|Il a fait une pause.
-narrateur|Plus tard, la pluie devient fine.
-papa|On va chercher le pain ?
-maman|Prenez le sac. Il est près de la porte.
-enfant-m|Oui. Le pain chaud.
-narrateur|Aniss et papa marchent sous le ciel gris.
-narrateur|Les gouttes font des ronds dans les flaques.
-narrateur|La boulangerie sent le beurre et la farine.
-narrateur|La file est longue.
-narrateur|Aniss sent ses pieds bouger.
-narrateur|Son ventre se serre un peu.
-enfant-m|C'est trop. J'attends. Je suis fâché.
-papa|Tu te souviens, Aniss ?
-papa|Tu peux souffler. Tu peux faire une pause.
-narrateur|Aniss s'assoit sur le banc, près de papa.
-narrateur|Il souffle, long et doux.
+          <t>narrateur|Aniss veut la tour, maintenant.
+enfant-m|Tout de suite !
+narrateur|Il pose les cubes trop vite.
+narrateur|La tour penche, puis tombe.
+narrateur|Son ventre reste serré.
+narrateur|Le sourire ne revient pas.
+enfant-m|Oh.
+narrateur|Aniss s'assoit près du bois.
+narrateur|Il pose les mains sur ses genoux.
+narrateur|Il souffle, un filet d'air.
+narrateur|L'air sort, long.
 narrateur|Il fait une pause.
-narrateur|Ses pieds se posent.
-enfant-m|Je souffle. Je fais une pause.
-papa|Bravo. Tu as repris, calme.
-narrateur|La file avance.
-narrateur|Le pain arrive, encore tiède.</t>
+papa|Tu restes près de nous, Aniss ?
+enfant-m|Je reste ici, papa ?
+papa|On s'assoit, puis on regarde.
+enfant-m|D'accord.
+narrateur|Aniss reste un moment, les mains ouvertes.
+narrateur|Sa poitrine descend, plus lente.
+papa|Merci, Aniss.
+narrateur|Papa a vu les deux, près des cubes.
+maman|Le bois est tiède, sous les doigts.
+enfant-m|Il est chaud.
+narrateur|Aniss reprend un cube, sans se presser.
+enfant-m|Sans me presser.
+papa|Il tient, là ?
+enfant-m|Oui, là.
+narrateur|La tour est petite.
+narrateur|Elle tient sur le bois.
+maman|Tes mains sont au chaud, Aniss ?
+enfant-m|Un peu, maman.
+enfant-m|On va au pain ?
+maman|Le sac est près de la porte ?
+enfant-m|Oui, maman.
+papa|Tu prends le sac, Aniss ?
+enfant-m|Oui, papa.
+narrateur|Aniss glisse la main sur le bois.
+enfant-m|Le petit point.
+papa|Il brille, là ?
+enfant-m|Oui, là.
+narrateur|Aniss pose les mains sur le bois.
+narrateur|Il reste, sans se presser.</t>
         </is>
       </c>
       <c r="AX4" t="inlineStr">
         <is>
-          <t>pluie,boulangerie</t>
+          <t>cubes</t>
         </is>
       </c>
     </row>
@@ -1789,17 +1812,17 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Aniss tient le pain encore tiède. Le papier craque un peu entre ses mains. Tu as attendu. Tu as soufflé. Le pain est chaud, papa. On rentre le montrer à maman ? Oui. Ils marchent. La pluie est fine. Aniss serre le pain contre son manteau. La maison n'est plus très loin.</t>
+          <t>Ils sortent vers la rue. La porte de la boulangerie s'ouvre. Le pain, maintenant ! Aniss avance trop vite. La file ne bouge pas. Le pain tiède est là, très près. Je le prends ! Aniss tend la main trop vite. Son ventre se serre. Oh. Aniss refuse de foncer. Il s'arrête net. Il souffle, un filet d'air. Il reste près de papa. Personne ne parle, un moment. Au bord du bois, un éclat de comptoir luit. Là, sur le bois. J'attends, papa ? Papa ne dit rien, d'abord. Il reste à la même hauteur. Tu l'entends, la file ? Oui, papa. La clochette a sonné, Aniss ? Oui, maman. La file avance, un pas. Aniss hoche la tête, sans se presser. Tu sens le pain, Aniss ? Oui, papa. Le papier est près du bois ? Oui, maman. Papa tend le pain, très tiède. Aniss pose les deux mains dessus. Le pain tient, Aniss ? Oui, papa. Un rayon passe sur le comptoir. Il allume le bois.</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Aniss tient le pain encore tiède. Le papier craque un peu entre ses mains. Tu as attendu. Tu as soufflé. Le pain est chaud, papa. On rentre le montrer à maman ? Oui. Ils marchent. La pluie est fine. Aniss serre le pain contre son manteau. La maison n'est plus très loin.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Ils sortent vers la rue. La porte de la boulangerie s'ouvre. Le pain, maintenant ! Aniss avance trop vite. La file ne bouge pas. Le pain tiède est là, très près. Je le prends ! Aniss tend la main trop vite. Son ventre se serre. Oh. Aniss refuse de foncer. Il s'arrête net. Il souffle, un filet d'air. Il reste près de papa. Personne ne parle, un moment. Au bord du bois, un &lt;emphasis level="moderate"&gt;éclat de comptoir&lt;/emphasis&gt; luit. Là, sur le bois. J'attends, papa ? Papa ne dit rien, d'abord. Il reste à la même hauteur. Tu l'entends, la file ? Oui, papa. La clochette a sonné, Aniss ? Oui, maman. La file avance, un pas. Aniss hoche la tête, sans se presser. Tu sens le pain, Aniss ? Oui, papa. Le papier est près du bois ? Oui, maman. Papa tend le pain, très tiède. Aniss pose les deux mains dessus. Le pain tient, Aniss ? Oui, papa. Un rayon passe sur le comptoir. Il allume le bois.&lt;/prosody&gt;&lt;break time="420ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>Yanis tient le pain. Papa sourit. [pause]</t>
+          <t>Ils sortent vers la rue. La porte de la boulangerie s'ouvre. Le pain, maintenant ! Aniss avance trop vite. La file ne bouge pas. Le pain tiède est là, très près. Je le prends ! Aniss tend la main trop vite. Son ventre se serre. Oh. Aniss refuse de foncer. Il s'arrête net. Il souffle, un filet d'air. Il reste près de papa. Personne ne parle, un moment. Au bord du bois, un &lt;emphasis&gt;éclat de comptoir&lt;/emphasis&gt; luit. Là, sur le bois. J'attends, papa ? Papa ne dit rien, d'abord. Il reste à la même hauteur. Tu l'entends, la file ? Oui, papa. La clochette a sonné, Aniss ? Oui, maman. La file avance, un pas. Aniss hoche la tête, sans se presser. Tu sens le pain, Aniss ? Oui, papa. Le papier est près du bois ? Oui, maman. Papa tend le pain, très tiède. Aniss pose les deux mains dessus. Le pain tient, Aniss ? Oui, papa. Un rayon passe sur le comptoir. Il allume le bois. [pause]</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr"/>
@@ -1846,7 +1869,7 @@
         </is>
       </c>
       <c r="Y5" s="2" t="n">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="Z5" s="2" t="inlineStr">
         <is>
@@ -1854,10 +1877,10 @@
         </is>
       </c>
       <c r="AA5" s="2" t="n">
-        <v>0.96</v>
+        <v>1</v>
       </c>
       <c r="AB5" s="2" t="n">
-        <v>1.12</v>
+        <v>1.1</v>
       </c>
       <c r="AC5" s="2" t="inlineStr">
         <is>
@@ -1878,28 +1901,32 @@
       <c r="AG5" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="AH5" s="2" t="inlineStr"/>
+      <c r="AH5" s="2" t="inlineStr">
+        <is>
+          <t>éclat de comptoir</t>
+        </is>
+      </c>
       <c r="AI5" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ5" s="2" t="n">
-        <v>450</v>
+        <v>420</v>
       </c>
       <c r="AK5" s="2" t="n">
-        <v>280</v>
+        <v>250</v>
       </c>
       <c r="AL5" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>lively</t>
         </is>
       </c>
       <c r="AM5" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>dynamic</t>
         </is>
       </c>
       <c r="AN5" s="2" t="n">
-        <v>0.333</v>
+        <v>0.37</v>
       </c>
       <c r="AO5" s="2" t="inlineStr"/>
       <c r="AP5" s="2" t="inlineStr">
@@ -1908,10 +1935,10 @@
         </is>
       </c>
       <c r="AQ5" s="2" t="n">
-        <v>0.96</v>
+        <v>1</v>
       </c>
       <c r="AR5" s="2" t="n">
-        <v>0.96</v>
+        <v>1</v>
       </c>
       <c r="AS5" s="2" t="n">
         <v>100</v>
@@ -1922,23 +1949,54 @@
       <c r="AU5" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="AV5" s="2" t="inlineStr"/>
+      <c r="AV5" s="2" t="inlineStr">
+        <is>
+          <t>arc=action; intention=entraîner; emotion=élan puis prudence; intensite=2; destinataire=enfant; sous_texte=pain_maintenant_il_souffle_il_reste; tempo=vif puis posé; sourire=léger; respiration=courte</t>
+        </is>
+      </c>
       <c r="AW5" t="inlineStr">
         <is>
-          <t>narrateur|Aniss tient le pain encore tiède.
-narrateur|Le papier craque un peu entre ses mains.
-papa|Tu as attendu. Tu as soufflé.
-enfant-m|Le pain est chaud, papa.
-papa|On rentre le montrer à maman ?
-enfant-m|Oui.
-narrateur|Ils marchent. La pluie est fine.
-narrateur|Aniss serre le pain contre son manteau.
-narrateur|La maison n'est plus très loin.</t>
+          <t>narrateur|Ils sortent vers la rue.
+narrateur|La porte de la boulangerie s'ouvre.
+enfant-m|Le pain, maintenant !
+narrateur|Aniss avance trop vite.
+narrateur|La file ne bouge pas.
+narrateur|Le pain tiède est là, très près.
+enfant-m|Je le prends !
+narrateur|Aniss tend la main trop vite.
+narrateur|Son ventre se serre.
+enfant-m|Oh.
+narrateur|Aniss refuse de foncer.
+narrateur|Il s'arrête net.
+narrateur|Il souffle, un filet d'air.
+narrateur|Il reste près de papa.
+narrateur|Personne ne parle, un moment.
+narrateur|Au bord du bois, un éclat de comptoir luit.
+enfant-m|Là, sur le bois.
+enfant-m|J'attends, papa ?
+narrateur|Papa ne dit rien, d'abord.
+narrateur|Il reste à la même hauteur.
+papa|Tu l'entends, la file ?
+enfant-m|Oui, papa.
+maman|La clochette a sonné, Aniss ?
+enfant-m|Oui, maman.
+narrateur|La file avance, un pas.
+narrateur|Aniss hoche la tête, sans se presser.
+papa|Tu sens le pain, Aniss ?
+enfant-m|Oui, papa.
+maman|Le papier est près du bois ?
+enfant-m|Oui, maman.
+narrateur|Papa tend le pain, très tiède.
+narrateur|Aniss pose les deux mains dessus.
+papa|Le pain tient, Aniss ?
+enfant-m|Oui, papa.
+maman|Un rayon passe sur le comptoir.
+enfant-m|Il allume le bois.</t>
         </is>
       </c>
       <c r="AX5" t="inlineStr">
         <is>
-          <t>pluie,papier</t>
+          <t>boulangerie</t>
         </is>
       </c>
     </row>
@@ -1965,17 +2023,17 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>J'ai soufflé. J'ai fait une pause. Bravo, Aniss. Le pain est là. Vous voilà. Ça sent bon, tout le salon.</t>
+          <t>Ils restent près du comptoir. Le pain a eu son tour, Aniss ? Oui, maman. Tu souffles un peu ? Oui, papa. Aniss souffle, un filet d'air. Le pain sent bon. Tu le sens, le pain ? Oui, maman. Le papier reste un peu, à plat. Il a tenu, sur le bois. La rue est calme, sous les mains. Le papier fait une petite ombre. On y revient, après. Un éclat de comptoir tient sur le bois.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>J'ai soufflé. J'ai fait une pause. Bravo, Aniss. Le pain est là. Vous voilà. Ça sent bon, tout le salon.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Ils restent près du comptoir. Le pain a eu son tour, Aniss ? Oui, maman. Tu souffles un peu ? Oui, papa. Aniss souffle, un filet d'air. Le pain sent bon. Tu le sens, le pain ? Oui, maman. Le papier reste un peu, à plat. Il a tenu, sur le bois. La rue est calme, sous les mains. Le papier fait une petite ombre. On y revient, après. Un &lt;emphasis level="moderate"&gt;éclat de comptoir&lt;/emphasis&gt; tient sur le bois.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>&lt;lower-pitch&gt;&lt;soft&gt;L'histoire est finie.&lt;/soft&gt;&lt;/lower-pitch&gt; [pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Ils restent près du comptoir. Le pain a eu son tour, Aniss ? Oui, maman. Tu souffles un peu ? Oui, papa. Aniss souffle, un filet d'air. Le pain sent bon. Tu le sens, le pain ? Oui, maman. Le papier reste un peu, à plat. Il a tenu, sur le bois. La rue est calme, sous les mains. Le papier fait une petite ombre. On y revient, après. Un &lt;emphasis&gt;éclat de comptoir&lt;/emphasis&gt; tient sur le bois.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr"/>
@@ -2022,18 +2080,18 @@
         </is>
       </c>
       <c r="Y6" s="2" t="n">
-        <v>136</v>
+        <v>118</v>
       </c>
       <c r="Z6" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>slow</t>
         </is>
       </c>
       <c r="AA6" s="2" t="n">
-        <v>0.92</v>
+        <v>0.85</v>
       </c>
       <c r="AB6" s="2" t="n">
-        <v>1.2</v>
+        <v>1.28</v>
       </c>
       <c r="AC6" s="2" t="inlineStr">
         <is>
@@ -2042,12 +2100,12 @@
       </c>
       <c r="AD6" s="2" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>-2st</t>
         </is>
       </c>
       <c r="AE6" s="2" t="inlineStr">
         <is>
-          <t>lower-pitch</t>
+          <t>low-pitch</t>
         </is>
       </c>
       <c r="AF6" s="2" t="inlineStr">
@@ -2056,17 +2114,21 @@
         </is>
       </c>
       <c r="AG6" s="2" t="n">
-        <v>-2</v>
-      </c>
-      <c r="AH6" s="2" t="inlineStr"/>
+        <v>-3</v>
+      </c>
+      <c r="AH6" s="2" t="inlineStr">
+        <is>
+          <t>éclat de comptoir</t>
+        </is>
+      </c>
       <c r="AI6" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ6" s="2" t="n">
-        <v>600</v>
+        <v>900</v>
       </c>
       <c r="AK6" s="2" t="n">
-        <v>280</v>
+        <v>340</v>
       </c>
       <c r="AL6" s="2" t="inlineStr">
         <is>
@@ -2075,11 +2137,11 @@
       </c>
       <c r="AM6" s="2" t="inlineStr">
         <is>
-          <t>fall</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN6" s="2" t="n">
-        <v>0.333</v>
+        <v>0.31</v>
       </c>
       <c r="AO6" s="2" t="inlineStr"/>
       <c r="AP6" s="2" t="inlineStr">
@@ -2088,27 +2150,42 @@
         </is>
       </c>
       <c r="AQ6" s="2" t="n">
-        <v>0.92</v>
+        <v>0.85</v>
       </c>
       <c r="AR6" s="2" t="n">
-        <v>0.92</v>
+        <v>0.85</v>
       </c>
       <c r="AS6" s="2" t="n">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="AT6" s="2" t="n">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="AU6" s="2" t="n">
-        <v>8</v>
-      </c>
-      <c r="AV6" s="2" t="inlineStr"/>
+        <v>12</v>
+      </c>
+      <c r="AV6" s="2" t="inlineStr">
+        <is>
+          <t>arc=retour; intention=refermer; emotion=tendresse_et_fierté_calme; intensite=1; destinataire=enfant; sous_texte=l_eclat_du_debut_tient_sur_le_bois; tempo=posé; sourire=léger; respiration=ample</t>
+        </is>
+      </c>
       <c r="AW6" t="inlineStr">
         <is>
-          <t>enfant-m|J'ai soufflé. J'ai fait une pause.
-papa|Bravo, Aniss.
-maman|Le pain est là. Vous voilà.
-maman|Ça sent bon, tout le salon.</t>
+          <t>narrateur|Ils restent près du comptoir.
+maman|Le pain a eu son tour, Aniss ?
+enfant-m|Oui, maman.
+papa|Tu souffles un peu ?
+enfant-m|Oui, papa.
+narrateur|Aniss souffle, un filet d'air.
+enfant-m|Le pain sent bon.
+maman|Tu le sens, le pain ?
+enfant-m|Oui, maman.
+papa|Le papier reste un peu, à plat.
+enfant-m|Il a tenu, sur le bois.
+narrateur|La rue est calme, sous les mains.
+narrateur|Le papier fait une petite ombre.
+enfant-m|On y revient, après.
+narrateur|Un éclat de comptoir tient sur le bois.</t>
         </is>
       </c>
     </row>
@@ -2129,7 +2206,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A7"/>
+  <dimension ref="A1:A8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -2179,6 +2256,13 @@
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
         <is>
           <t>F-NAR-008 récit, pas une leçon en puces</t>
         </is>

</xml_diff>